<commit_message>
fix: improved area chairman info
</commit_message>
<xml_diff>
--- a/samples/ra/26-27/Royal Arch Official Visit Matrix 2026 - 2027 MF V5 04082026.xlsx
+++ b/samples/ra/26-27/Royal Arch Official Visit Matrix 2026 - 2027 MF V5 04082026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kpturner/github/square_ov/samples/ra/26-27/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BCE495C-8049-D147-92C3-062968F85437}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95FB973F-0FA1-834A-9352-41240D49A55F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="30520" yWindow="29360" windowWidth="34360" windowHeight="19800" tabRatio="500" xr2:uid="{FA0C5B21-D744-41D8-A854-64181BC35FE8}"/>
   </bookViews>
@@ -71,7 +71,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1378" uniqueCount="520">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1382" uniqueCount="527">
   <si>
     <t>Name</t>
   </si>
@@ -422,9 +422,6 @@
   </si>
   <si>
     <t>Ward</t>
-  </si>
-  <si>
-    <t>RA Area Chair</t>
   </si>
   <si>
     <t>OV No.</t>
@@ -1662,6 +1659,30 @@
   <si>
     <t>Hilton MBE, RN</t>
   </si>
+  <si>
+    <t xml:space="preserve">Charles </t>
+  </si>
+  <si>
+    <t>McGeoch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">David </t>
+  </si>
+  <si>
+    <t>Conway-Holland</t>
+  </si>
+  <si>
+    <t>Michael</t>
+  </si>
+  <si>
+    <t>Geddes</t>
+  </si>
+  <si>
+    <t>Brett</t>
+  </si>
+  <si>
+    <t>Clark</t>
+  </si>
 </sst>
 </file>
 
@@ -1670,7 +1691,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yy"/>
   </numFmts>
-  <fonts count="49" x14ac:knownFonts="1">
+  <fonts count="50" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -2000,6 +2021,13 @@
       <sz val="11"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="77">
@@ -2811,7 +2839,7 @@
     <xf numFmtId="0" fontId="1" fillId="36" borderId="20" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="41" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="208">
+  <cellXfs count="210">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
@@ -3377,6 +3405,12 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="44">
@@ -3884,7 +3918,7 @@
     </row>
     <row r="2" spans="1:51" ht="14" x14ac:dyDescent="0.15">
       <c r="E2" s="13" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F2" s="30">
         <v>1</v>
@@ -3991,103 +4025,103 @@
         <v>0</v>
       </c>
       <c r="F3" s="45" t="s">
+        <v>120</v>
+      </c>
+      <c r="G3" s="49" t="s">
+        <v>125</v>
+      </c>
+      <c r="H3" s="50" t="s">
+        <v>126</v>
+      </c>
+      <c r="I3" s="49" t="s">
+        <v>127</v>
+      </c>
+      <c r="J3" s="51" t="s">
+        <v>128</v>
+      </c>
+      <c r="K3" s="52" t="s">
+        <v>129</v>
+      </c>
+      <c r="L3" s="51" t="s">
         <v>121</v>
       </c>
-      <c r="G3" s="49" t="s">
-        <v>126</v>
-      </c>
-      <c r="H3" s="50" t="s">
-        <v>127</v>
-      </c>
-      <c r="I3" s="49" t="s">
-        <v>128</v>
-      </c>
-      <c r="J3" s="51" t="s">
-        <v>129</v>
-      </c>
-      <c r="K3" s="52" t="s">
+      <c r="M3" s="51" t="s">
+        <v>131</v>
+      </c>
+      <c r="N3" s="51" t="s">
         <v>130</v>
       </c>
-      <c r="L3" s="51" t="s">
-        <v>122</v>
-      </c>
-      <c r="M3" s="51" t="s">
+      <c r="O3" s="52" t="s">
         <v>132</v>
       </c>
-      <c r="N3" s="51" t="s">
-        <v>131</v>
-      </c>
-      <c r="O3" s="52" t="s">
+      <c r="P3" s="52" t="s">
         <v>133</v>
       </c>
-      <c r="P3" s="52" t="s">
+      <c r="Q3" s="85" t="s">
+        <v>219</v>
+      </c>
+      <c r="R3" s="52" t="s">
+        <v>218</v>
+      </c>
+      <c r="S3" s="51" t="s">
         <v>134</v>
       </c>
-      <c r="Q3" s="85" t="s">
-        <v>220</v>
-      </c>
-      <c r="R3" s="52" t="s">
-        <v>219</v>
-      </c>
-      <c r="S3" s="51" t="s">
+      <c r="T3" s="52" t="s">
         <v>135</v>
       </c>
-      <c r="T3" s="52" t="s">
+      <c r="U3" s="51" t="s">
         <v>136</v>
       </c>
-      <c r="U3" s="51" t="s">
+      <c r="V3" s="52" t="s">
+        <v>145</v>
+      </c>
+      <c r="W3" s="52" t="s">
         <v>137</v>
       </c>
-      <c r="V3" s="52" t="s">
-        <v>146</v>
-      </c>
-      <c r="W3" s="52" t="s">
+      <c r="X3" s="54" t="s">
+        <v>165</v>
+      </c>
+      <c r="Y3" s="51" t="s">
         <v>138</v>
       </c>
-      <c r="X3" s="54" t="s">
-        <v>166</v>
-      </c>
-      <c r="Y3" s="51" t="s">
+      <c r="Z3" s="52" t="s">
         <v>139</v>
-      </c>
-      <c r="Z3" s="52" t="s">
-        <v>140</v>
       </c>
       <c r="AA3" s="52" t="s">
         <v>4</v>
       </c>
       <c r="AB3" s="52" t="s">
+        <v>140</v>
+      </c>
+      <c r="AC3" s="53" t="s">
+        <v>122</v>
+      </c>
+      <c r="AD3" s="51" t="s">
         <v>141</v>
       </c>
-      <c r="AC3" s="53" t="s">
+      <c r="AE3" s="51" t="s">
+        <v>142</v>
+      </c>
+      <c r="AF3" s="52" t="s">
+        <v>143</v>
+      </c>
+      <c r="AG3" s="51" t="s">
+        <v>144</v>
+      </c>
+      <c r="AH3" s="51" t="s">
         <v>123</v>
       </c>
-      <c r="AD3" s="51" t="s">
-        <v>142</v>
-      </c>
-      <c r="AE3" s="51" t="s">
-        <v>143</v>
-      </c>
-      <c r="AF3" s="52" t="s">
-        <v>144</v>
-      </c>
-      <c r="AG3" s="51" t="s">
-        <v>145</v>
-      </c>
-      <c r="AH3" s="51" t="s">
+      <c r="AI3" s="51" t="s">
         <v>124</v>
       </c>
-      <c r="AI3" s="51" t="s">
-        <v>125</v>
-      </c>
       <c r="AJ3" s="52" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="AK3" s="51" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="AL3" s="60" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="AX3" s="12"/>
     </row>
@@ -4215,7 +4249,7 @@
         <v>7</v>
       </c>
       <c r="I5" s="80" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="J5" s="81" t="s">
         <v>8</v>
@@ -4227,13 +4261,13 @@
         <v>12</v>
       </c>
       <c r="M5" s="81" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="N5" s="81" t="s">
         <v>8</v>
       </c>
       <c r="O5" s="80" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="P5" s="80" t="s">
         <v>6</v>
@@ -4242,7 +4276,7 @@
         <v>11</v>
       </c>
       <c r="R5" s="80" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="S5" s="81" t="s">
         <v>9</v>
@@ -4251,19 +4285,19 @@
         <v>6</v>
       </c>
       <c r="U5" s="81" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="V5" s="80" t="s">
         <v>6</v>
       </c>
       <c r="W5" s="80" t="s">
+        <v>151</v>
+      </c>
+      <c r="X5" s="82" t="s">
+        <v>166</v>
+      </c>
+      <c r="Y5" s="81" t="s">
         <v>152</v>
-      </c>
-      <c r="X5" s="82" t="s">
-        <v>167</v>
-      </c>
-      <c r="Y5" s="81" t="s">
-        <v>153</v>
       </c>
       <c r="Z5" s="80" t="s">
         <v>10</v>
@@ -4275,10 +4309,10 @@
         <v>5</v>
       </c>
       <c r="AC5" s="65" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="AD5" s="81" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="AE5" s="81" t="s">
         <v>3</v>
@@ -4287,13 +4321,13 @@
         <v>11</v>
       </c>
       <c r="AG5" s="81" t="s">
+        <v>154</v>
+      </c>
+      <c r="AH5" s="81" t="s">
         <v>155</v>
       </c>
-      <c r="AH5" s="81" t="s">
+      <c r="AI5" s="81" t="s">
         <v>156</v>
-      </c>
-      <c r="AI5" s="81" t="s">
-        <v>157</v>
       </c>
       <c r="AJ5" s="80" t="s">
         <v>13</v>
@@ -4418,7 +4452,7 @@
         <v>26</v>
       </c>
       <c r="E7" s="42" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F7" s="58">
         <f t="shared" ref="F7:AL7" si="0">COUNTIF(F10:F62,"YES")</f>
@@ -4662,7 +4696,7 @@
     </row>
     <row r="9" spans="1:51" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="E9" s="44" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F9" s="7"/>
       <c r="G9" s="16"/>
@@ -4694,7 +4728,7 @@
       <c r="AI9" s="16"/>
       <c r="AJ9" s="16"/>
       <c r="AM9" s="44" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="10" spans="1:51" s="20" customFormat="1" x14ac:dyDescent="0.2">
@@ -4773,7 +4807,7 @@
     </row>
     <row r="11" spans="1:51" s="20" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A11" s="31" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B11" s="32" t="s">
         <v>31</v>
@@ -4854,7 +4888,7 @@
         <v>33</v>
       </c>
       <c r="B12" s="78" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>112</v>
@@ -5189,7 +5223,7 @@
         <v>61</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D16" s="4" t="s">
         <v>47</v>
@@ -5384,7 +5418,7 @@
         <v>52</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>53</v>
@@ -5466,7 +5500,7 @@
         <v>55</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>56</v>
@@ -5546,7 +5580,7 @@
         <v>43</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>59</v>
@@ -5624,7 +5658,7 @@
         <v>60</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>110</v>
@@ -5707,10 +5741,10 @@
         <v>63</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D22" s="10" t="s">
         <v>64</v>
@@ -5790,7 +5824,7 @@
         <v>65</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>67</v>
@@ -5873,7 +5907,7 @@
         <v>65</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>68</v>
@@ -5914,7 +5948,7 @@
         <v>30</v>
       </c>
       <c r="X24" s="205" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="Y24" s="21"/>
       <c r="Z24" s="21"/>
@@ -5956,10 +5990,10 @@
         <v>65</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D25" s="4" t="s">
         <v>66</v>
@@ -6039,10 +6073,10 @@
         <v>69</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D26" s="4" t="s">
         <v>71</v>
@@ -6067,7 +6101,7 @@
       <c r="O26" s="21"/>
       <c r="P26" s="127"/>
       <c r="Q26" s="88" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="R26" s="22"/>
       <c r="S26" s="102" t="s">
@@ -6120,7 +6154,7 @@
         <v>72</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>74</v>
@@ -6169,7 +6203,7 @@
       </c>
       <c r="AA27" s="21"/>
       <c r="AB27" s="21" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="AC27" s="126" t="s">
         <v>30</v>
@@ -6205,7 +6239,7 @@
         <v>76</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>77</v>
@@ -6338,7 +6372,7 @@
         <v>30</v>
       </c>
       <c r="AB29" s="21" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="AC29" s="126" t="s">
         <v>30</v>
@@ -6374,10 +6408,10 @@
         <v>84</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D30" s="4" t="s">
         <v>85</v>
@@ -6459,7 +6493,7 @@
         <v>86</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C31" s="3" t="s">
         <v>88</v>
@@ -6497,7 +6531,7 @@
       </c>
       <c r="R31" s="21"/>
       <c r="S31" s="194" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="T31" s="98" t="s">
         <v>30</v>
@@ -6558,10 +6592,10 @@
         <v>90</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D32" s="4" t="s">
         <v>91</v>
@@ -6587,7 +6621,7 @@
       </c>
       <c r="P32" s="21"/>
       <c r="Q32" s="193" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="R32" s="22"/>
       <c r="S32" s="98" t="s">
@@ -6601,7 +6635,7 @@
       <c r="W32" s="21"/>
       <c r="X32" s="21"/>
       <c r="Y32" s="194" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="Z32" s="21"/>
       <c r="AA32" s="21" t="s">
@@ -6646,10 +6680,10 @@
         <v>92</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D33" s="4" t="s">
         <v>93</v>
@@ -6676,7 +6710,7 @@
       </c>
       <c r="P33" s="21"/>
       <c r="Q33" s="126" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="R33" s="22"/>
       <c r="S33" s="21"/>
@@ -6729,10 +6763,10 @@
         <v>94</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D34" s="4" t="s">
         <v>95</v>
@@ -6744,7 +6778,7 @@
       <c r="F34" s="130"/>
       <c r="G34" s="21"/>
       <c r="H34" s="130" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="I34" s="21"/>
       <c r="J34" s="21"/>
@@ -6822,7 +6856,7 @@
         <v>96</v>
       </c>
       <c r="B35" s="77" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="C35" s="3" t="s">
         <v>116</v>
@@ -6901,10 +6935,10 @@
         <v>96</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D36" s="4" t="s">
         <v>98</v>
@@ -6980,10 +7014,10 @@
         <v>96</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D37" s="4" t="s">
         <v>98</v>
@@ -7062,10 +7096,10 @@
         <v>96</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D38" s="6" t="s">
         <v>98</v>
@@ -7142,7 +7176,7 @@
         <v>61</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D39" s="6" t="s">
         <v>98</v>
@@ -7178,10 +7212,10 @@
         <v>30</v>
       </c>
       <c r="W39" s="21" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="X39" s="106" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="Y39" s="21"/>
       <c r="Z39" s="106" t="s">
@@ -7215,7 +7249,7 @@
         <v>100</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="C40" s="5" t="s">
         <v>101</v>
@@ -7299,7 +7333,7 @@
         <v>97</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D41" s="6" t="s">
         <v>104</v>
@@ -7382,10 +7416,10 @@
         <v>103</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D42" s="6" t="s">
         <v>104</v>
@@ -7405,7 +7439,7 @@
       <c r="K42" s="103"/>
       <c r="L42" s="21"/>
       <c r="M42" s="204" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="N42" s="21"/>
       <c r="O42" s="100"/>
@@ -7468,10 +7502,10 @@
         <v>103</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D43" s="6" t="s">
         <v>104</v>
@@ -7488,7 +7522,7 @@
       </c>
       <c r="J43" s="21"/>
       <c r="K43" s="202" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="L43" s="21"/>
       <c r="M43" s="21"/>
@@ -7527,7 +7561,7 @@
       </c>
       <c r="AF43" s="99"/>
       <c r="AG43" s="203" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="AH43" s="21"/>
       <c r="AI43" s="21"/>
@@ -7554,7 +7588,7 @@
         <v>105</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C44" s="5" t="s">
         <v>106</v>
@@ -7637,10 +7671,10 @@
         <v>108</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D45" s="6" t="s">
         <v>109</v>
@@ -7722,10 +7756,10 @@
         <v>108</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D46" s="6" t="s">
         <v>109</v>
@@ -7805,10 +7839,10 @@
         <v>108</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D47" s="6" t="s">
         <v>109</v>
@@ -7837,7 +7871,7 @@
       <c r="O47" s="21"/>
       <c r="P47" s="21"/>
       <c r="Q47" s="126" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="R47" s="22"/>
       <c r="S47" s="21"/>
@@ -7856,7 +7890,7 @@
         <v>30</v>
       </c>
       <c r="AB47" s="200" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="AC47" s="126" t="s">
         <v>30</v>
@@ -7864,7 +7898,7 @@
       <c r="AD47" s="21"/>
       <c r="AE47" s="21"/>
       <c r="AF47" s="98" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="AG47" s="103" t="s">
         <v>30</v>
@@ -7894,7 +7928,7 @@
         <v>108</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C48" s="5" t="s">
         <v>31</v>
@@ -7912,7 +7946,7 @@
       <c r="G48" s="21"/>
       <c r="H48" s="21"/>
       <c r="I48" s="98" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="J48" s="103"/>
       <c r="K48" s="21"/>
@@ -7981,10 +8015,10 @@
         <v>108</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D49" s="6" t="s">
         <v>109</v>
@@ -8000,7 +8034,7 @@
       <c r="H49" s="103"/>
       <c r="I49" s="21"/>
       <c r="J49" s="21" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="K49" s="21"/>
       <c r="L49" s="21"/>
@@ -8064,10 +8098,10 @@
         <v>108</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D50" s="6" t="s">
         <v>109</v>
@@ -8147,10 +8181,10 @@
         <v>108</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C51" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D51" s="6" t="s">
         <v>109</v>
@@ -8234,10 +8268,10 @@
         <v>108</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="D52" s="6" t="s">
         <v>109</v>
@@ -8319,10 +8353,10 @@
         <v>108</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D53" s="6" t="s">
         <v>109</v>
@@ -8349,7 +8383,7 @@
       </c>
       <c r="P53" s="21"/>
       <c r="Q53" s="126" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="R53" s="22" t="s">
         <v>30</v>
@@ -8404,10 +8438,10 @@
         <v>108</v>
       </c>
       <c r="B54" s="68" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C54" s="68" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D54" s="69" t="s">
         <v>109</v>
@@ -8452,7 +8486,7 @@
       <c r="Y54" s="103"/>
       <c r="Z54" s="21"/>
       <c r="AA54" s="98" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="AB54" s="21"/>
       <c r="AC54" s="126" t="s">
@@ -8487,10 +8521,10 @@
         <v>108</v>
       </c>
       <c r="B55" s="74" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C55" s="56" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D55" s="69" t="s">
         <v>109</v>
@@ -8572,10 +8606,10 @@
         <v>108</v>
       </c>
       <c r="B56" s="74" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C56" s="56" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D56" s="69" t="s">
         <v>109</v>
@@ -8654,13 +8688,15 @@
     </row>
     <row r="57" spans="1:51" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A57" s="75" t="s">
-        <v>160</v>
-      </c>
-      <c r="B57" s="76"/>
-      <c r="C57" s="76"/>
-      <c r="D57" s="76" t="s">
-        <v>117</v>
-      </c>
+        <v>159</v>
+      </c>
+      <c r="B57" s="208" t="s">
+        <v>519</v>
+      </c>
+      <c r="C57" s="76" t="s">
+        <v>520</v>
+      </c>
+      <c r="D57" s="76"/>
       <c r="E57" s="43">
         <f t="shared" si="4"/>
         <v>4</v>
@@ -8712,18 +8748,20 @@
       </c>
       <c r="AN57" s="12" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve"> </v>
+        <v>Charles  McGeoch</v>
       </c>
     </row>
     <row r="58" spans="1:51" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A58" s="71" t="s">
-        <v>161</v>
-      </c>
-      <c r="B58" s="72"/>
-      <c r="C58" s="72"/>
-      <c r="D58" s="72" t="s">
-        <v>117</v>
-      </c>
+        <v>160</v>
+      </c>
+      <c r="B58" s="209" t="s">
+        <v>521</v>
+      </c>
+      <c r="C58" s="72" t="s">
+        <v>522</v>
+      </c>
+      <c r="D58" s="72"/>
       <c r="E58" s="73">
         <f t="shared" si="4"/>
         <v>6</v>
@@ -8779,18 +8817,20 @@
       </c>
       <c r="AN58" s="12" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve"> </v>
+        <v>David  Conway-Holland</v>
       </c>
     </row>
     <row r="59" spans="1:51" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A59" s="59" t="s">
-        <v>162</v>
-      </c>
-      <c r="B59" s="26"/>
-      <c r="C59" s="26"/>
-      <c r="D59" s="26" t="s">
-        <v>117</v>
-      </c>
+        <v>161</v>
+      </c>
+      <c r="B59" s="26" t="s">
+        <v>523</v>
+      </c>
+      <c r="C59" s="26" t="s">
+        <v>524</v>
+      </c>
+      <c r="D59" s="26"/>
       <c r="E59" s="43">
         <f t="shared" si="4"/>
         <v>7</v>
@@ -8848,18 +8888,16 @@
       </c>
       <c r="AN59" s="12" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve"> </v>
+        <v>Michael Geddes</v>
       </c>
     </row>
     <row r="60" spans="1:51" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A60" s="59" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B60" s="26"/>
       <c r="C60" s="26"/>
-      <c r="D60" s="26" t="s">
-        <v>117</v>
-      </c>
+      <c r="D60" s="26"/>
       <c r="E60" s="43">
         <f t="shared" si="4"/>
         <v>8</v>
@@ -8924,13 +8962,15 @@
     </row>
     <row r="61" spans="1:51" s="28" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A61" s="59" t="s">
-        <v>164</v>
-      </c>
-      <c r="B61" s="26"/>
-      <c r="C61" s="27"/>
-      <c r="D61" s="26" t="s">
-        <v>117</v>
-      </c>
+        <v>163</v>
+      </c>
+      <c r="B61" s="26" t="s">
+        <v>43</v>
+      </c>
+      <c r="C61" s="27" t="s">
+        <v>518</v>
+      </c>
+      <c r="D61" s="26"/>
       <c r="E61" s="43">
         <f t="shared" si="4"/>
         <v>5</v>
@@ -8984,7 +9024,7 @@
       </c>
       <c r="AN61" s="12" t="str">
         <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
+        <v>David Hilton MBE, RN</v>
       </c>
       <c r="AY61" s="12"/>
     </row>
@@ -8992,11 +9032,13 @@
       <c r="A62" s="59" t="s">
         <v>111</v>
       </c>
-      <c r="B62" s="26"/>
-      <c r="C62" s="26"/>
-      <c r="D62" s="26" t="s">
-        <v>117</v>
-      </c>
+      <c r="B62" s="26" t="s">
+        <v>525</v>
+      </c>
+      <c r="C62" s="26" t="s">
+        <v>526</v>
+      </c>
+      <c r="D62" s="26"/>
       <c r="E62" s="43">
         <f t="shared" si="4"/>
         <v>7</v>
@@ -9054,7 +9096,7 @@
       </c>
       <c r="AN62" s="12" t="str">
         <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
+        <v>Brett Clark</v>
       </c>
     </row>
   </sheetData>
@@ -9086,37 +9128,37 @@
   <sheetData>
     <row r="3" spans="4:19" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D3" s="124" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="E3" s="116" t="s">
+        <v>221</v>
+      </c>
+      <c r="F3" s="116" t="s">
+        <v>493</v>
+      </c>
+      <c r="G3" s="116" t="s">
         <v>222</v>
       </c>
-      <c r="F3" s="116" t="s">
-        <v>494</v>
-      </c>
-      <c r="G3" s="116" t="s">
+      <c r="H3" s="116" t="s">
         <v>223</v>
       </c>
-      <c r="H3" s="116" t="s">
+      <c r="I3" s="116" t="s">
         <v>224</v>
       </c>
-      <c r="I3" s="116" t="s">
+      <c r="J3" s="116" t="s">
         <v>225</v>
       </c>
-      <c r="J3" s="116" t="s">
+      <c r="K3" s="116" t="s">
         <v>226</v>
       </c>
-      <c r="K3" s="116" t="s">
+      <c r="L3" s="116" t="s">
         <v>227</v>
       </c>
-      <c r="L3" s="116" t="s">
+      <c r="M3" s="116" t="s">
         <v>228</v>
       </c>
-      <c r="M3" s="116" t="s">
+      <c r="N3" s="116" t="s">
         <v>229</v>
-      </c>
-      <c r="N3" s="116" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="4" spans="4:19" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -9127,27 +9169,27 @@
         <v>42</v>
       </c>
       <c r="F4" s="117" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="G4" s="118"/>
       <c r="H4" s="117" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I4" s="117" t="s">
         <v>43</v>
       </c>
       <c r="J4" s="117" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="K4" s="118"/>
       <c r="L4" s="117" t="s">
+        <v>233</v>
+      </c>
+      <c r="M4" s="117" t="s">
         <v>234</v>
       </c>
-      <c r="M4" s="117" t="s">
+      <c r="N4" s="117" t="s">
         <v>235</v>
-      </c>
-      <c r="N4" s="117" t="s">
-        <v>236</v>
       </c>
     </row>
     <row r="5" spans="4:19" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -9158,36 +9200,36 @@
         <v>61</v>
       </c>
       <c r="F5" s="150" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="G5" s="151"/>
       <c r="H5" s="150" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="I5" s="150" t="s">
         <v>61</v>
       </c>
       <c r="J5" s="150" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="K5" s="151"/>
       <c r="L5" s="150" t="s">
+        <v>238</v>
+      </c>
+      <c r="M5" s="150" t="s">
         <v>239</v>
       </c>
-      <c r="M5" s="150" t="s">
+      <c r="N5" s="150" t="s">
         <v>240</v>
       </c>
-      <c r="N5" s="150" t="s">
-        <v>241</v>
-      </c>
       <c r="P5" s="196" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="R5" s="166" t="s">
         <v>14</v>
       </c>
       <c r="S5" s="181" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
     </row>
     <row r="6" spans="4:19" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -9198,35 +9240,35 @@
         <v>49</v>
       </c>
       <c r="F6" s="153" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="G6" s="154"/>
       <c r="H6" s="153" t="s">
+        <v>242</v>
+      </c>
+      <c r="I6" s="153" t="s">
         <v>243</v>
       </c>
-      <c r="I6" s="153" t="s">
+      <c r="J6" s="153" t="s">
+        <v>232</v>
+      </c>
+      <c r="K6" s="153" t="s">
         <v>244</v>
       </c>
-      <c r="J6" s="153" t="s">
-        <v>233</v>
-      </c>
-      <c r="K6" s="153" t="s">
+      <c r="L6" s="153" t="s">
         <v>245</v>
       </c>
-      <c r="L6" s="153" t="s">
+      <c r="M6" s="153" t="s">
         <v>246</v>
       </c>
-      <c r="M6" s="153" t="s">
+      <c r="N6" s="153" t="s">
         <v>247</v>
       </c>
-      <c r="N6" s="153" t="s">
-        <v>248</v>
-      </c>
       <c r="R6" s="166" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="S6" s="178" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
     </row>
     <row r="7" spans="4:19" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -9234,36 +9276,36 @@
         <v>52</v>
       </c>
       <c r="E7" s="117" t="s">
+        <v>248</v>
+      </c>
+      <c r="F7" s="117" t="s">
         <v>249</v>
-      </c>
-      <c r="F7" s="117" t="s">
-        <v>250</v>
       </c>
       <c r="G7" s="118"/>
       <c r="H7" s="117" t="s">
+        <v>250</v>
+      </c>
+      <c r="I7" s="117" t="s">
         <v>251</v>
       </c>
-      <c r="I7" s="117" t="s">
+      <c r="J7" s="117" t="s">
+        <v>232</v>
+      </c>
+      <c r="K7" s="117" t="s">
         <v>252</v>
-      </c>
-      <c r="J7" s="117" t="s">
-        <v>233</v>
-      </c>
-      <c r="K7" s="117" t="s">
-        <v>253</v>
       </c>
       <c r="L7" s="118"/>
       <c r="M7" s="117" t="s">
+        <v>253</v>
+      </c>
+      <c r="N7" s="117" t="s">
         <v>254</v>
       </c>
-      <c r="N7" s="117" t="s">
-        <v>255</v>
-      </c>
       <c r="R7" s="168" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="S7" s="179" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
     </row>
     <row r="8" spans="4:19" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -9271,38 +9313,38 @@
         <v>55</v>
       </c>
       <c r="E8" s="117" t="s">
+        <v>255</v>
+      </c>
+      <c r="F8" s="117" t="s">
         <v>256</v>
-      </c>
-      <c r="F8" s="117" t="s">
-        <v>257</v>
       </c>
       <c r="G8" s="118"/>
       <c r="H8" s="117" t="s">
+        <v>257</v>
+      </c>
+      <c r="I8" s="117" t="s">
         <v>258</v>
       </c>
-      <c r="I8" s="117" t="s">
+      <c r="J8" s="117" t="s">
+        <v>232</v>
+      </c>
+      <c r="K8" s="117" t="s">
         <v>259</v>
       </c>
-      <c r="J8" s="117" t="s">
-        <v>233</v>
-      </c>
-      <c r="K8" s="117" t="s">
+      <c r="L8" s="117" t="s">
         <v>260</v>
       </c>
-      <c r="L8" s="117" t="s">
+      <c r="M8" s="117" t="s">
         <v>261</v>
       </c>
-      <c r="M8" s="117" t="s">
+      <c r="N8" s="117" t="s">
         <v>262</v>
       </c>
-      <c r="N8" s="117" t="s">
-        <v>263</v>
-      </c>
       <c r="R8" s="167" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="S8" s="180" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
     </row>
     <row r="9" spans="4:19" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -9313,37 +9355,37 @@
         <v>43</v>
       </c>
       <c r="F9" s="117" t="s">
+        <v>263</v>
+      </c>
+      <c r="G9" s="117" t="s">
         <v>264</v>
       </c>
-      <c r="G9" s="117" t="s">
+      <c r="H9" s="117" t="s">
         <v>265</v>
-      </c>
-      <c r="H9" s="117" t="s">
-        <v>266</v>
       </c>
       <c r="I9" s="118" t="s">
         <v>43</v>
       </c>
       <c r="J9" s="117" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="K9" s="117" t="s">
+        <v>266</v>
+      </c>
+      <c r="L9" s="117" t="s">
         <v>267</v>
       </c>
-      <c r="L9" s="117" t="s">
+      <c r="M9" s="117" t="s">
         <v>268</v>
       </c>
-      <c r="M9" s="117" t="s">
+      <c r="N9" s="117" t="s">
         <v>269</v>
       </c>
-      <c r="N9" s="117" t="s">
-        <v>270</v>
-      </c>
       <c r="R9" s="168" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="S9" s="179" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="10" spans="4:19" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -9351,30 +9393,30 @@
         <v>60</v>
       </c>
       <c r="E10" s="117" t="s">
+        <v>270</v>
+      </c>
+      <c r="F10" s="117" t="s">
         <v>271</v>
-      </c>
-      <c r="F10" s="117" t="s">
-        <v>272</v>
       </c>
       <c r="G10" s="118"/>
       <c r="H10" s="117" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="I10" s="118" t="s">
         <v>70</v>
       </c>
       <c r="J10" s="117" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="K10" s="118"/>
       <c r="L10" s="117" t="s">
+        <v>273</v>
+      </c>
+      <c r="M10" s="117" t="s">
         <v>274</v>
       </c>
-      <c r="M10" s="117" t="s">
+      <c r="N10" s="117" t="s">
         <v>275</v>
-      </c>
-      <c r="N10" s="117" t="s">
-        <v>276</v>
       </c>
     </row>
     <row r="11" spans="4:19" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -9382,32 +9424,32 @@
         <v>63</v>
       </c>
       <c r="E11" s="153" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F11" s="153" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="G11" s="154"/>
       <c r="H11" s="153" t="s">
+        <v>277</v>
+      </c>
+      <c r="I11" s="153" t="s">
+        <v>258</v>
+      </c>
+      <c r="J11" s="153" t="s">
+        <v>232</v>
+      </c>
+      <c r="K11" s="153" t="s">
         <v>278</v>
       </c>
-      <c r="I11" s="153" t="s">
-        <v>259</v>
-      </c>
-      <c r="J11" s="153" t="s">
-        <v>233</v>
-      </c>
-      <c r="K11" s="153" t="s">
+      <c r="L11" s="153" t="s">
         <v>279</v>
       </c>
-      <c r="L11" s="153" t="s">
+      <c r="M11" s="153" t="s">
         <v>280</v>
       </c>
-      <c r="M11" s="153" t="s">
+      <c r="N11" s="153" t="s">
         <v>281</v>
-      </c>
-      <c r="N11" s="153" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="12" spans="4:19" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -9415,32 +9457,32 @@
         <v>65</v>
       </c>
       <c r="E12" s="117" t="s">
+        <v>282</v>
+      </c>
+      <c r="F12" s="117" t="s">
         <v>283</v>
-      </c>
-      <c r="F12" s="117" t="s">
-        <v>284</v>
       </c>
       <c r="G12" s="118"/>
       <c r="H12" s="117" t="s">
+        <v>284</v>
+      </c>
+      <c r="I12" s="117" t="s">
+        <v>243</v>
+      </c>
+      <c r="J12" s="117" t="s">
+        <v>232</v>
+      </c>
+      <c r="K12" s="117" t="s">
         <v>285</v>
       </c>
-      <c r="I12" s="117" t="s">
-        <v>244</v>
-      </c>
-      <c r="J12" s="117" t="s">
-        <v>233</v>
-      </c>
-      <c r="K12" s="117" t="s">
+      <c r="L12" s="117" t="s">
         <v>286</v>
       </c>
-      <c r="L12" s="117" t="s">
+      <c r="M12" s="117" t="s">
         <v>287</v>
       </c>
-      <c r="M12" s="117" t="s">
+      <c r="N12" s="117" t="s">
         <v>288</v>
-      </c>
-      <c r="N12" s="117" t="s">
-        <v>289</v>
       </c>
     </row>
     <row r="13" spans="4:19" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -9448,30 +9490,30 @@
         <v>65</v>
       </c>
       <c r="E13" s="117" t="s">
+        <v>289</v>
+      </c>
+      <c r="F13" s="117" t="s">
         <v>290</v>
-      </c>
-      <c r="F13" s="117" t="s">
-        <v>291</v>
       </c>
       <c r="G13" s="118"/>
       <c r="H13" s="117" t="s">
+        <v>291</v>
+      </c>
+      <c r="I13" s="117" t="s">
         <v>292</v>
       </c>
-      <c r="I13" s="117" t="s">
-        <v>293</v>
-      </c>
       <c r="J13" s="117" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="K13" s="118"/>
       <c r="L13" s="117" t="s">
+        <v>293</v>
+      </c>
+      <c r="M13" s="117" t="s">
         <v>294</v>
       </c>
-      <c r="M13" s="117" t="s">
+      <c r="N13" s="117" t="s">
         <v>295</v>
-      </c>
-      <c r="N13" s="117" t="s">
-        <v>296</v>
       </c>
     </row>
     <row r="14" spans="4:19" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -9479,32 +9521,32 @@
         <v>65</v>
       </c>
       <c r="E14" s="117" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F14" s="117" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="G14" s="118"/>
       <c r="H14" s="117" t="s">
+        <v>297</v>
+      </c>
+      <c r="I14" s="117" t="s">
         <v>298</v>
       </c>
-      <c r="I14" s="117" t="s">
+      <c r="J14" s="117" t="s">
+        <v>232</v>
+      </c>
+      <c r="K14" s="117" t="s">
         <v>299</v>
       </c>
-      <c r="J14" s="117" t="s">
-        <v>233</v>
-      </c>
-      <c r="K14" s="117" t="s">
+      <c r="L14" s="117" t="s">
         <v>300</v>
       </c>
-      <c r="L14" s="117" t="s">
+      <c r="M14" s="117" t="s">
         <v>301</v>
       </c>
-      <c r="M14" s="117" t="s">
+      <c r="N14" s="117" t="s">
         <v>302</v>
-      </c>
-      <c r="N14" s="117" t="s">
-        <v>303</v>
       </c>
     </row>
     <row r="15" spans="4:19" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -9512,32 +9554,32 @@
         <v>69</v>
       </c>
       <c r="E15" s="117" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F15" s="117" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="G15" s="118"/>
       <c r="H15" s="117" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="I15" s="117" t="s">
+        <v>304</v>
+      </c>
+      <c r="J15" s="117" t="s">
+        <v>232</v>
+      </c>
+      <c r="K15" s="117" t="s">
         <v>305</v>
       </c>
-      <c r="J15" s="117" t="s">
-        <v>233</v>
-      </c>
-      <c r="K15" s="117" t="s">
+      <c r="L15" s="117" t="s">
         <v>306</v>
       </c>
-      <c r="L15" s="117" t="s">
+      <c r="M15" s="117" t="s">
         <v>307</v>
       </c>
-      <c r="M15" s="117" t="s">
+      <c r="N15" s="117" t="s">
         <v>308</v>
-      </c>
-      <c r="N15" s="117" t="s">
-        <v>309</v>
       </c>
     </row>
     <row r="16" spans="4:19" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -9545,32 +9587,32 @@
         <v>72</v>
       </c>
       <c r="E16" s="117" t="s">
+        <v>309</v>
+      </c>
+      <c r="F16" s="117" t="s">
         <v>310</v>
-      </c>
-      <c r="F16" s="117" t="s">
-        <v>311</v>
       </c>
       <c r="G16" s="118"/>
       <c r="H16" s="117" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="I16" s="117" t="s">
         <v>73</v>
       </c>
       <c r="J16" s="117" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="K16" s="117" t="s">
+        <v>311</v>
+      </c>
+      <c r="L16" s="117" t="s">
         <v>312</v>
       </c>
-      <c r="L16" s="117" t="s">
+      <c r="M16" s="117" t="s">
         <v>313</v>
       </c>
-      <c r="M16" s="117" t="s">
+      <c r="N16" s="117" t="s">
         <v>314</v>
-      </c>
-      <c r="N16" s="117" t="s">
-        <v>315</v>
       </c>
     </row>
     <row r="17" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -9578,35 +9620,35 @@
         <v>76</v>
       </c>
       <c r="E17" s="117" t="s">
+        <v>315</v>
+      </c>
+      <c r="F17" s="117" t="s">
         <v>316</v>
-      </c>
-      <c r="F17" s="117" t="s">
-        <v>317</v>
       </c>
       <c r="G17" s="118"/>
       <c r="H17" s="117" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="I17" s="118" t="s">
         <v>43</v>
       </c>
       <c r="J17" s="117" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="K17" s="117" t="s">
+        <v>318</v>
+      </c>
+      <c r="L17" s="117" t="s">
         <v>319</v>
       </c>
-      <c r="L17" s="117" t="s">
+      <c r="M17" s="117" t="s">
         <v>320</v>
       </c>
-      <c r="M17" s="117" t="s">
+      <c r="N17" s="117" t="s">
         <v>321</v>
       </c>
-      <c r="N17" s="117" t="s">
-        <v>322</v>
-      </c>
       <c r="P17" s="195" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
     </row>
     <row r="18" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -9617,27 +9659,27 @@
         <v>80</v>
       </c>
       <c r="F18" s="117" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="G18" s="118"/>
       <c r="H18" s="117" t="s">
+        <v>323</v>
+      </c>
+      <c r="I18" s="117" t="s">
         <v>324</v>
       </c>
-      <c r="I18" s="117" t="s">
-        <v>325</v>
-      </c>
       <c r="J18" s="117" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="K18" s="118"/>
       <c r="L18" s="117" t="s">
+        <v>325</v>
+      </c>
+      <c r="M18" s="117" t="s">
         <v>326</v>
       </c>
-      <c r="M18" s="117" t="s">
+      <c r="N18" s="117" t="s">
         <v>327</v>
-      </c>
-      <c r="N18" s="117" t="s">
-        <v>328</v>
       </c>
     </row>
     <row r="19" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -9645,30 +9687,30 @@
         <v>84</v>
       </c>
       <c r="E19" s="117" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F19" s="117" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G19" s="118"/>
       <c r="H19" s="117" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="I19" s="117" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="J19" s="117" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="K19" s="118"/>
       <c r="L19" s="117" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="M19" s="121" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="N19" s="117" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
     </row>
     <row r="20" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -9676,35 +9718,35 @@
         <v>86</v>
       </c>
       <c r="E20" s="117" t="s">
+        <v>328</v>
+      </c>
+      <c r="F20" s="117" t="s">
         <v>329</v>
-      </c>
-      <c r="F20" s="117" t="s">
-        <v>330</v>
       </c>
       <c r="G20" s="118"/>
       <c r="H20" s="117" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="I20" s="117" t="s">
         <v>87</v>
       </c>
       <c r="J20" s="117" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="K20" s="117" t="s">
+        <v>331</v>
+      </c>
+      <c r="L20" s="117" t="s">
         <v>332</v>
       </c>
-      <c r="L20" s="117" t="s">
+      <c r="M20" s="117" t="s">
         <v>333</v>
       </c>
-      <c r="M20" s="117" t="s">
+      <c r="N20" s="117" t="s">
         <v>334</v>
       </c>
-      <c r="N20" s="117" t="s">
-        <v>335</v>
-      </c>
       <c r="P20" s="195" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
     </row>
     <row r="21" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -9712,32 +9754,32 @@
         <v>90</v>
       </c>
       <c r="E21" s="117" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F21" s="117" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="G21" s="118"/>
       <c r="H21" s="117" t="s">
+        <v>336</v>
+      </c>
+      <c r="I21" s="118" t="s">
+        <v>494</v>
+      </c>
+      <c r="J21" s="117" t="s">
+        <v>232</v>
+      </c>
+      <c r="K21" s="117" t="s">
         <v>337</v>
       </c>
-      <c r="I21" s="118" t="s">
-        <v>495</v>
-      </c>
-      <c r="J21" s="117" t="s">
-        <v>233</v>
-      </c>
-      <c r="K21" s="117" t="s">
+      <c r="L21" s="117" t="s">
         <v>338</v>
       </c>
-      <c r="L21" s="117" t="s">
+      <c r="M21" s="117" t="s">
         <v>339</v>
       </c>
-      <c r="M21" s="117" t="s">
+      <c r="N21" s="117" t="s">
         <v>340</v>
-      </c>
-      <c r="N21" s="117" t="s">
-        <v>341</v>
       </c>
     </row>
     <row r="22" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -9745,30 +9787,30 @@
         <v>92</v>
       </c>
       <c r="E22" s="117" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="F22" s="117" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="G22" s="118"/>
       <c r="H22" s="117" t="s">
+        <v>342</v>
+      </c>
+      <c r="I22" s="117" t="s">
         <v>343</v>
       </c>
-      <c r="I22" s="117" t="s">
-        <v>344</v>
-      </c>
       <c r="J22" s="117" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="K22" s="118"/>
       <c r="L22" s="117" t="s">
+        <v>344</v>
+      </c>
+      <c r="M22" s="117" t="s">
         <v>345</v>
       </c>
-      <c r="M22" s="117" t="s">
+      <c r="N22" s="117" t="s">
         <v>346</v>
-      </c>
-      <c r="N22" s="117" t="s">
-        <v>347</v>
       </c>
     </row>
     <row r="23" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -9776,32 +9818,32 @@
         <v>94</v>
       </c>
       <c r="E23" s="157" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F23" s="157" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="G23" s="158"/>
       <c r="H23" s="157" t="s">
+        <v>348</v>
+      </c>
+      <c r="I23" s="157" t="s">
         <v>349</v>
       </c>
-      <c r="I23" s="157" t="s">
+      <c r="J23" s="157" t="s">
+        <v>232</v>
+      </c>
+      <c r="K23" s="157" t="s">
         <v>350</v>
       </c>
-      <c r="J23" s="157" t="s">
-        <v>233</v>
-      </c>
-      <c r="K23" s="157" t="s">
+      <c r="L23" s="157" t="s">
         <v>351</v>
       </c>
-      <c r="L23" s="157" t="s">
+      <c r="M23" s="157" t="s">
         <v>352</v>
       </c>
-      <c r="M23" s="157" t="s">
+      <c r="N23" s="157" t="s">
         <v>353</v>
-      </c>
-      <c r="N23" s="157" t="s">
-        <v>354</v>
       </c>
     </row>
     <row r="24" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -9809,32 +9851,32 @@
         <v>96</v>
       </c>
       <c r="E24" s="160" t="s">
+        <v>354</v>
+      </c>
+      <c r="F24" s="160" t="s">
         <v>355</v>
-      </c>
-      <c r="F24" s="160" t="s">
-        <v>356</v>
       </c>
       <c r="G24" s="161"/>
       <c r="H24" s="160" t="s">
+        <v>356</v>
+      </c>
+      <c r="I24" s="160" t="s">
         <v>357</v>
       </c>
-      <c r="I24" s="160" t="s">
+      <c r="J24" s="160" t="s">
+        <v>232</v>
+      </c>
+      <c r="K24" s="160" t="s">
         <v>358</v>
       </c>
-      <c r="J24" s="160" t="s">
-        <v>233</v>
-      </c>
-      <c r="K24" s="160" t="s">
+      <c r="L24" s="160" t="s">
         <v>359</v>
       </c>
-      <c r="L24" s="160" t="s">
+      <c r="M24" s="160" t="s">
         <v>360</v>
       </c>
-      <c r="M24" s="160" t="s">
+      <c r="N24" s="160" t="s">
         <v>361</v>
-      </c>
-      <c r="N24" s="160" t="s">
-        <v>362</v>
       </c>
     </row>
     <row r="25" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -9842,30 +9884,30 @@
         <v>96</v>
       </c>
       <c r="E25" s="117" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F25" s="117" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="G25" s="118"/>
       <c r="H25" s="117" t="s">
+        <v>363</v>
+      </c>
+      <c r="I25" s="117" t="s">
         <v>364</v>
       </c>
-      <c r="I25" s="117" t="s">
-        <v>365</v>
-      </c>
       <c r="J25" s="117" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="K25" s="118"/>
       <c r="L25" s="117" t="s">
+        <v>365</v>
+      </c>
+      <c r="M25" s="117" t="s">
         <v>366</v>
       </c>
-      <c r="M25" s="117" t="s">
+      <c r="N25" s="117" t="s">
         <v>367</v>
-      </c>
-      <c r="N25" s="117" t="s">
-        <v>368</v>
       </c>
     </row>
     <row r="26" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -9873,30 +9915,30 @@
         <v>96</v>
       </c>
       <c r="E26" s="157" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F26" s="157" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="G26" s="158"/>
       <c r="H26" s="157" t="s">
+        <v>369</v>
+      </c>
+      <c r="I26" s="157" t="s">
+        <v>324</v>
+      </c>
+      <c r="J26" s="157" t="s">
         <v>370</v>
-      </c>
-      <c r="I26" s="157" t="s">
-        <v>325</v>
-      </c>
-      <c r="J26" s="157" t="s">
-        <v>371</v>
       </c>
       <c r="K26" s="158"/>
       <c r="L26" s="157" t="s">
+        <v>371</v>
+      </c>
+      <c r="M26" s="157" t="s">
         <v>372</v>
       </c>
-      <c r="M26" s="157" t="s">
+      <c r="N26" s="157" t="s">
         <v>373</v>
-      </c>
-      <c r="N26" s="157" t="s">
-        <v>374</v>
       </c>
     </row>
     <row r="27" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -9904,32 +9946,32 @@
         <v>96</v>
       </c>
       <c r="E27" s="150" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="F27" s="150" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="G27" s="151"/>
       <c r="H27" s="150" t="s">
+        <v>375</v>
+      </c>
+      <c r="I27" s="150" t="s">
         <v>376</v>
       </c>
-      <c r="I27" s="150" t="s">
+      <c r="J27" s="150" t="s">
+        <v>232</v>
+      </c>
+      <c r="K27" s="150" t="s">
         <v>377</v>
       </c>
-      <c r="J27" s="150" t="s">
-        <v>233</v>
-      </c>
-      <c r="K27" s="150" t="s">
+      <c r="L27" s="150" t="s">
         <v>378</v>
       </c>
-      <c r="L27" s="150" t="s">
+      <c r="M27" s="150" t="s">
         <v>379</v>
       </c>
-      <c r="M27" s="150" t="s">
+      <c r="N27" s="150" t="s">
         <v>380</v>
-      </c>
-      <c r="N27" s="150" t="s">
-        <v>381</v>
       </c>
     </row>
     <row r="28" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -9940,29 +9982,29 @@
         <v>61</v>
       </c>
       <c r="F28" s="117" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="G28" s="118"/>
       <c r="H28" s="117" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="I28" s="117" t="s">
         <v>61</v>
       </c>
       <c r="J28" s="117" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="K28" s="117" t="s">
+        <v>382</v>
+      </c>
+      <c r="L28" s="117" t="s">
         <v>383</v>
       </c>
-      <c r="L28" s="117" t="s">
+      <c r="M28" s="117" t="s">
         <v>384</v>
       </c>
-      <c r="M28" s="117" t="s">
+      <c r="N28" s="117" t="s">
         <v>385</v>
-      </c>
-      <c r="N28" s="117" t="s">
-        <v>386</v>
       </c>
     </row>
     <row r="29" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -9970,32 +10012,32 @@
         <v>100</v>
       </c>
       <c r="E29" s="117" t="s">
+        <v>386</v>
+      </c>
+      <c r="F29" s="117" t="s">
         <v>387</v>
-      </c>
-      <c r="F29" s="117" t="s">
-        <v>388</v>
       </c>
       <c r="G29" s="118"/>
       <c r="H29" s="117" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="I29" s="117" t="s">
         <v>81</v>
       </c>
       <c r="J29" s="117" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="K29" s="117" t="s">
+        <v>389</v>
+      </c>
+      <c r="L29" s="117" t="s">
+        <v>389</v>
+      </c>
+      <c r="M29" s="117" t="s">
         <v>390</v>
       </c>
-      <c r="L29" s="117" t="s">
-        <v>390</v>
-      </c>
-      <c r="M29" s="117" t="s">
+      <c r="N29" s="117" t="s">
         <v>391</v>
-      </c>
-      <c r="N29" s="117" t="s">
-        <v>392</v>
       </c>
     </row>
     <row r="30" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -10006,29 +10048,29 @@
         <v>97</v>
       </c>
       <c r="F30" s="157" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="G30" s="158"/>
       <c r="H30" s="157" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="I30" s="157" t="s">
         <v>97</v>
       </c>
       <c r="J30" s="157" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="K30" s="157" t="s">
+        <v>394</v>
+      </c>
+      <c r="L30" s="157" t="s">
         <v>395</v>
       </c>
-      <c r="L30" s="157" t="s">
+      <c r="M30" s="157" t="s">
         <v>396</v>
       </c>
-      <c r="M30" s="157" t="s">
+      <c r="N30" s="157" t="s">
         <v>397</v>
-      </c>
-      <c r="N30" s="157" t="s">
-        <v>398</v>
       </c>
     </row>
     <row r="31" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -10036,32 +10078,32 @@
         <v>103</v>
       </c>
       <c r="E31" s="117" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="F31" s="117" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="G31" s="118"/>
       <c r="H31" s="117" t="s">
+        <v>399</v>
+      </c>
+      <c r="I31" s="117" t="s">
         <v>400</v>
       </c>
-      <c r="I31" s="117" t="s">
+      <c r="J31" s="117" t="s">
+        <v>232</v>
+      </c>
+      <c r="K31" s="117" t="s">
         <v>401</v>
       </c>
-      <c r="J31" s="117" t="s">
-        <v>233</v>
-      </c>
-      <c r="K31" s="117" t="s">
+      <c r="L31" s="117" t="s">
         <v>402</v>
       </c>
-      <c r="L31" s="117" t="s">
+      <c r="M31" s="117" t="s">
         <v>403</v>
       </c>
-      <c r="M31" s="117" t="s">
+      <c r="N31" s="117" t="s">
         <v>404</v>
-      </c>
-      <c r="N31" s="117" t="s">
-        <v>405</v>
       </c>
     </row>
     <row r="32" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -10069,32 +10111,32 @@
         <v>103</v>
       </c>
       <c r="E32" s="160" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="F32" s="160" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G32" s="161"/>
       <c r="H32" s="160" t="s">
+        <v>406</v>
+      </c>
+      <c r="I32" s="160" t="s">
         <v>407</v>
       </c>
-      <c r="I32" s="160" t="s">
+      <c r="J32" s="160" t="s">
+        <v>232</v>
+      </c>
+      <c r="K32" s="160" t="s">
         <v>408</v>
       </c>
-      <c r="J32" s="160" t="s">
-        <v>233</v>
-      </c>
-      <c r="K32" s="160" t="s">
+      <c r="L32" s="160" t="s">
         <v>409</v>
       </c>
-      <c r="L32" s="160" t="s">
+      <c r="M32" s="160" t="s">
         <v>410</v>
       </c>
-      <c r="M32" s="160" t="s">
+      <c r="N32" s="160" t="s">
         <v>411</v>
-      </c>
-      <c r="N32" s="160" t="s">
-        <v>412</v>
       </c>
     </row>
     <row r="33" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -10102,32 +10144,32 @@
         <v>105</v>
       </c>
       <c r="E33" s="117" t="s">
+        <v>486</v>
+      </c>
+      <c r="F33" s="117" t="s">
         <v>487</v>
-      </c>
-      <c r="F33" s="117" t="s">
-        <v>488</v>
       </c>
       <c r="G33" s="118"/>
       <c r="H33" s="117" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="I33" s="117" t="s">
         <v>99</v>
       </c>
       <c r="J33" s="117" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="K33" s="117" t="s">
+        <v>489</v>
+      </c>
+      <c r="L33" s="117" t="s">
         <v>490</v>
       </c>
-      <c r="L33" s="117" t="s">
+      <c r="M33" s="117" t="s">
         <v>491</v>
       </c>
-      <c r="M33" s="117" t="s">
+      <c r="N33" s="117" t="s">
         <v>492</v>
-      </c>
-      <c r="N33" s="117" t="s">
-        <v>493</v>
       </c>
     </row>
     <row r="34" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -10135,32 +10177,32 @@
         <v>108</v>
       </c>
       <c r="E34" s="153" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F34" s="153" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="G34" s="154"/>
       <c r="H34" s="153" t="s">
+        <v>413</v>
+      </c>
+      <c r="I34" s="153" t="s">
         <v>414</v>
       </c>
-      <c r="I34" s="153" t="s">
+      <c r="J34" s="153" t="s">
+        <v>232</v>
+      </c>
+      <c r="K34" s="153" t="s">
         <v>415</v>
       </c>
-      <c r="J34" s="153" t="s">
-        <v>233</v>
-      </c>
-      <c r="K34" s="153" t="s">
+      <c r="L34" s="153" t="s">
         <v>416</v>
       </c>
-      <c r="L34" s="153" t="s">
+      <c r="M34" s="153" t="s">
         <v>417</v>
       </c>
-      <c r="M34" s="153" t="s">
+      <c r="N34" s="153" t="s">
         <v>418</v>
-      </c>
-      <c r="N34" s="153" t="s">
-        <v>419</v>
       </c>
     </row>
     <row r="35" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -10168,32 +10210,32 @@
         <v>108</v>
       </c>
       <c r="E35" s="150" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F35" s="150" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="G35" s="151"/>
       <c r="H35" s="150" t="s">
+        <v>420</v>
+      </c>
+      <c r="I35" s="150" t="s">
         <v>421</v>
       </c>
-      <c r="I35" s="150" t="s">
+      <c r="J35" s="150" t="s">
+        <v>232</v>
+      </c>
+      <c r="K35" s="150" t="s">
         <v>422</v>
       </c>
-      <c r="J35" s="150" t="s">
-        <v>233</v>
-      </c>
-      <c r="K35" s="150" t="s">
+      <c r="L35" s="150" t="s">
         <v>423</v>
       </c>
-      <c r="L35" s="150" t="s">
+      <c r="M35" s="150" t="s">
         <v>424</v>
       </c>
-      <c r="M35" s="150" t="s">
+      <c r="N35" s="150" t="s">
         <v>425</v>
-      </c>
-      <c r="N35" s="150" t="s">
-        <v>426</v>
       </c>
     </row>
     <row r="36" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -10201,33 +10243,33 @@
         <v>108</v>
       </c>
       <c r="E36" s="157" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F36" s="157" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="G36" s="158"/>
       <c r="H36" s="157" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="I36" s="157" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="J36" s="157" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="K36" s="158"/>
       <c r="L36" s="157" t="s">
+        <v>428</v>
+      </c>
+      <c r="M36" s="157" t="s">
         <v>429</v>
       </c>
-      <c r="M36" s="157" t="s">
+      <c r="N36" s="157" t="s">
         <v>430</v>
       </c>
-      <c r="N36" s="157" t="s">
-        <v>431</v>
-      </c>
       <c r="P36" s="196" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
     </row>
     <row r="37" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -10235,32 +10277,32 @@
         <v>108</v>
       </c>
       <c r="E37" s="157" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F37" s="157" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="G37" s="158"/>
       <c r="H37" s="157" t="s">
+        <v>432</v>
+      </c>
+      <c r="I37" s="157" t="s">
         <v>433</v>
       </c>
-      <c r="I37" s="157" t="s">
+      <c r="J37" s="157" t="s">
+        <v>232</v>
+      </c>
+      <c r="K37" s="157" t="s">
         <v>434</v>
       </c>
-      <c r="J37" s="157" t="s">
-        <v>233</v>
-      </c>
-      <c r="K37" s="157" t="s">
+      <c r="L37" s="157" t="s">
         <v>435</v>
       </c>
-      <c r="L37" s="157" t="s">
+      <c r="M37" s="157" t="s">
         <v>436</v>
       </c>
-      <c r="M37" s="157" t="s">
+      <c r="N37" s="157" t="s">
         <v>437</v>
-      </c>
-      <c r="N37" s="157" t="s">
-        <v>438</v>
       </c>
     </row>
     <row r="38" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -10268,32 +10310,32 @@
         <v>108</v>
       </c>
       <c r="E38" s="170" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F38" s="170" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="G38" s="171"/>
       <c r="H38" s="170" t="s">
+        <v>439</v>
+      </c>
+      <c r="I38" s="170" t="s">
         <v>440</v>
       </c>
-      <c r="I38" s="170" t="s">
+      <c r="J38" s="170" t="s">
+        <v>232</v>
+      </c>
+      <c r="K38" s="170" t="s">
         <v>441</v>
       </c>
-      <c r="J38" s="170" t="s">
-        <v>233</v>
-      </c>
-      <c r="K38" s="170" t="s">
+      <c r="L38" s="170" t="s">
         <v>442</v>
       </c>
-      <c r="L38" s="170" t="s">
+      <c r="M38" s="170" t="s">
         <v>443</v>
       </c>
-      <c r="M38" s="170" t="s">
+      <c r="N38" s="170" t="s">
         <v>444</v>
-      </c>
-      <c r="N38" s="170" t="s">
-        <v>445</v>
       </c>
     </row>
     <row r="39" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -10301,35 +10343,35 @@
         <v>108</v>
       </c>
       <c r="E39" s="157" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F39" s="157" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="G39" s="158"/>
       <c r="H39" s="157" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="I39" s="157" t="s">
+        <v>446</v>
+      </c>
+      <c r="J39" s="157" t="s">
+        <v>232</v>
+      </c>
+      <c r="K39" s="157" t="s">
         <v>447</v>
       </c>
-      <c r="J39" s="157" t="s">
-        <v>233</v>
-      </c>
-      <c r="K39" s="157" t="s">
+      <c r="L39" s="157" t="s">
         <v>448</v>
       </c>
-      <c r="L39" s="157" t="s">
+      <c r="M39" s="157" t="s">
         <v>449</v>
       </c>
-      <c r="M39" s="157" t="s">
+      <c r="N39" s="157" t="s">
         <v>450</v>
       </c>
-      <c r="N39" s="157" t="s">
-        <v>451</v>
-      </c>
       <c r="P39" s="196" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
     </row>
     <row r="40" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -10337,30 +10379,30 @@
         <v>108</v>
       </c>
       <c r="E40" s="150" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F40" s="150" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="G40" s="151"/>
       <c r="H40" s="150" t="s">
+        <v>452</v>
+      </c>
+      <c r="I40" s="150" t="s">
         <v>453</v>
       </c>
-      <c r="I40" s="150" t="s">
-        <v>454</v>
-      </c>
       <c r="J40" s="150" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="K40" s="151"/>
       <c r="L40" s="150" t="s">
+        <v>454</v>
+      </c>
+      <c r="M40" s="150" t="s">
         <v>455</v>
       </c>
-      <c r="M40" s="150" t="s">
+      <c r="N40" s="150" t="s">
         <v>456</v>
-      </c>
-      <c r="N40" s="150" t="s">
-        <v>457</v>
       </c>
     </row>
     <row r="41" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -10368,35 +10410,35 @@
         <v>108</v>
       </c>
       <c r="E41" s="150" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F41" s="150" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="G41" s="151"/>
       <c r="H41" s="150" t="s">
+        <v>458</v>
+      </c>
+      <c r="I41" s="150" t="s">
         <v>459</v>
       </c>
-      <c r="I41" s="150" t="s">
+      <c r="J41" s="150" t="s">
+        <v>232</v>
+      </c>
+      <c r="K41" s="150" t="s">
         <v>460</v>
       </c>
-      <c r="J41" s="150" t="s">
-        <v>233</v>
-      </c>
-      <c r="K41" s="150" t="s">
+      <c r="L41" s="150" t="s">
         <v>461</v>
       </c>
-      <c r="L41" s="150" t="s">
+      <c r="M41" s="150" t="s">
         <v>462</v>
       </c>
-      <c r="M41" s="150" t="s">
+      <c r="N41" s="150" t="s">
         <v>463</v>
       </c>
-      <c r="N41" s="150" t="s">
-        <v>464</v>
-      </c>
       <c r="P41" s="201" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
     </row>
     <row r="42" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -10404,32 +10446,32 @@
         <v>108</v>
       </c>
       <c r="E42" s="117" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F42" s="117" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="G42" s="118"/>
       <c r="H42" s="117" t="s">
+        <v>291</v>
+      </c>
+      <c r="I42" s="117" t="s">
         <v>292</v>
       </c>
-      <c r="I42" s="117" t="s">
-        <v>293</v>
-      </c>
       <c r="J42" s="117" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="K42" s="117" t="s">
+        <v>465</v>
+      </c>
+      <c r="L42" s="117" t="s">
         <v>466</v>
       </c>
-      <c r="L42" s="117" t="s">
+      <c r="M42" s="117" t="s">
         <v>467</v>
       </c>
-      <c r="M42" s="117" t="s">
+      <c r="N42" s="117" t="s">
         <v>468</v>
-      </c>
-      <c r="N42" s="117" t="s">
-        <v>469</v>
       </c>
     </row>
     <row r="43" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -10437,32 +10479,32 @@
         <v>108</v>
       </c>
       <c r="E43" s="117" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F43" s="117" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="G43" s="118"/>
       <c r="H43" s="117" t="s">
+        <v>470</v>
+      </c>
+      <c r="I43" s="117" t="s">
+        <v>440</v>
+      </c>
+      <c r="J43" s="117" t="s">
+        <v>232</v>
+      </c>
+      <c r="K43" s="117" t="s">
         <v>471</v>
       </c>
-      <c r="I43" s="117" t="s">
-        <v>441</v>
-      </c>
-      <c r="J43" s="117" t="s">
-        <v>233</v>
-      </c>
-      <c r="K43" s="117" t="s">
+      <c r="L43" s="117" t="s">
         <v>472</v>
       </c>
-      <c r="L43" s="117" t="s">
+      <c r="M43" s="117" t="s">
         <v>473</v>
       </c>
-      <c r="M43" s="117" t="s">
+      <c r="N43" s="117" t="s">
         <v>474</v>
-      </c>
-      <c r="N43" s="117" t="s">
-        <v>475</v>
       </c>
     </row>
     <row r="44" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -10470,28 +10512,28 @@
         <v>108</v>
       </c>
       <c r="E44" s="117" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F44" s="117" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="G44" s="118"/>
       <c r="H44" s="117" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="I44" s="118"/>
       <c r="J44" s="117" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="K44" s="118"/>
       <c r="L44" s="117" t="s">
+        <v>477</v>
+      </c>
+      <c r="M44" s="117" t="s">
         <v>478</v>
       </c>
-      <c r="M44" s="117" t="s">
+      <c r="N44" s="117" t="s">
         <v>479</v>
-      </c>
-      <c r="N44" s="117" t="s">
-        <v>480</v>
       </c>
     </row>
     <row r="45" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -10499,32 +10541,32 @@
         <v>108</v>
       </c>
       <c r="E45" s="191" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="F45" s="191" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="G45" s="192"/>
       <c r="H45" s="191" t="s">
+        <v>481</v>
+      </c>
+      <c r="I45" s="191" t="s">
+        <v>324</v>
+      </c>
+      <c r="J45" s="191" t="s">
+        <v>232</v>
+      </c>
+      <c r="K45" s="191" t="s">
         <v>482</v>
       </c>
-      <c r="I45" s="191" t="s">
-        <v>325</v>
-      </c>
-      <c r="J45" s="191" t="s">
-        <v>233</v>
-      </c>
-      <c r="K45" s="191" t="s">
+      <c r="L45" s="191" t="s">
         <v>483</v>
       </c>
-      <c r="L45" s="191" t="s">
+      <c r="M45" s="191" t="s">
         <v>484</v>
       </c>
-      <c r="M45" s="191" t="s">
+      <c r="N45" s="191" t="s">
         <v>485</v>
-      </c>
-      <c r="N45" s="191" t="s">
-        <v>486</v>
       </c>
     </row>
     <row r="46" spans="4:16" x14ac:dyDescent="0.15">

</xml_diff>

<commit_message>
fix: more area chairman updates
</commit_message>
<xml_diff>
--- a/samples/ra/26-27/Royal Arch Official Visit Matrix 2026 - 2027 MF V5 04082026.xlsx
+++ b/samples/ra/26-27/Royal Arch Official Visit Matrix 2026 - 2027 MF V5 04082026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kpturner/github/square_ov/samples/ra/26-27/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95FB973F-0FA1-834A-9352-41240D49A55F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC4A4D1B-9B8E-9349-BF8C-1D3E8D833FA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30520" yWindow="29360" windowWidth="34360" windowHeight="19800" tabRatio="500" xr2:uid="{FA0C5B21-D744-41D8-A854-64181BC35FE8}"/>
+    <workbookView xWindow="30520" yWindow="29360" windowWidth="34360" windowHeight="19800" tabRatio="500" activeTab="1" xr2:uid="{FA0C5B21-D744-41D8-A854-64181BC35FE8}"/>
   </bookViews>
   <sheets>
     <sheet name="2026-2027 Official Visits" sheetId="1" r:id="rId1"/>
@@ -71,7 +71,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1382" uniqueCount="527">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1390" uniqueCount="530">
   <si>
     <t>Name</t>
   </si>
@@ -1163,9 +1163,6 @@
     <t>TJ</t>
   </si>
   <si>
-    <t>Jeremy</t>
-  </si>
-  <si>
     <t>01256 842021</t>
   </si>
   <si>
@@ -1666,22 +1663,34 @@
     <t>McGeoch</t>
   </si>
   <si>
-    <t xml:space="preserve">David </t>
-  </si>
-  <si>
-    <t>Conway-Holland</t>
-  </si>
-  <si>
     <t>Michael</t>
   </si>
   <si>
     <t>Geddes</t>
   </si>
   <si>
-    <t>Brett</t>
-  </si>
-  <si>
-    <t>Clark</t>
+    <t>Jerry</t>
+  </si>
+  <si>
+    <t>Nasser</t>
+  </si>
+  <si>
+    <t>Sharifi</t>
+  </si>
+  <si>
+    <t>Jordan</t>
+  </si>
+  <si>
+    <t>PPDepGSwdB</t>
+  </si>
+  <si>
+    <t>PPGReg</t>
+  </si>
+  <si>
+    <t>PPDepGDC</t>
+  </si>
+  <si>
+    <t>PPGSE</t>
   </si>
 </sst>
 </file>
@@ -4115,7 +4124,7 @@
         <v>124</v>
       </c>
       <c r="AJ3" s="52" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="AK3" s="51" t="s">
         <v>146</v>
@@ -5580,7 +5589,7 @@
         <v>43</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>59</v>
@@ -5948,7 +5957,7 @@
         <v>30</v>
       </c>
       <c r="X24" s="205" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="Y24" s="21"/>
       <c r="Z24" s="21"/>
@@ -6101,7 +6110,7 @@
       <c r="O26" s="21"/>
       <c r="P26" s="127"/>
       <c r="Q26" s="88" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="R26" s="22"/>
       <c r="S26" s="102" t="s">
@@ -6203,7 +6212,7 @@
       </c>
       <c r="AA27" s="21"/>
       <c r="AB27" s="21" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="AC27" s="126" t="s">
         <v>30</v>
@@ -6372,7 +6381,7 @@
         <v>30</v>
       </c>
       <c r="AB29" s="21" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="AC29" s="126" t="s">
         <v>30</v>
@@ -6531,7 +6540,7 @@
       </c>
       <c r="R31" s="21"/>
       <c r="S31" s="194" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="T31" s="98" t="s">
         <v>30</v>
@@ -6621,7 +6630,7 @@
       </c>
       <c r="P32" s="21"/>
       <c r="Q32" s="193" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="R32" s="22"/>
       <c r="S32" s="98" t="s">
@@ -6635,7 +6644,7 @@
       <c r="W32" s="21"/>
       <c r="X32" s="21"/>
       <c r="Y32" s="194" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="Z32" s="21"/>
       <c r="AA32" s="21" t="s">
@@ -6710,7 +6719,7 @@
       </c>
       <c r="P33" s="21"/>
       <c r="Q33" s="126" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="R33" s="22"/>
       <c r="S33" s="21"/>
@@ -6778,7 +6787,7 @@
       <c r="F34" s="130"/>
       <c r="G34" s="21"/>
       <c r="H34" s="130" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="I34" s="21"/>
       <c r="J34" s="21"/>
@@ -7212,10 +7221,10 @@
         <v>30</v>
       </c>
       <c r="W39" s="21" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="X39" s="106" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="Y39" s="21"/>
       <c r="Z39" s="106" t="s">
@@ -7249,7 +7258,7 @@
         <v>100</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="C40" s="5" t="s">
         <v>101</v>
@@ -7439,7 +7448,7 @@
       <c r="K42" s="103"/>
       <c r="L42" s="21"/>
       <c r="M42" s="204" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="N42" s="21"/>
       <c r="O42" s="100"/>
@@ -7522,7 +7531,7 @@
       </c>
       <c r="J43" s="21"/>
       <c r="K43" s="202" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="L43" s="21"/>
       <c r="M43" s="21"/>
@@ -7561,7 +7570,7 @@
       </c>
       <c r="AF43" s="99"/>
       <c r="AG43" s="203" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="AH43" s="21"/>
       <c r="AI43" s="21"/>
@@ -7588,7 +7597,7 @@
         <v>105</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="C44" s="5" t="s">
         <v>106</v>
@@ -7871,7 +7880,7 @@
       <c r="O47" s="21"/>
       <c r="P47" s="21"/>
       <c r="Q47" s="126" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="R47" s="22"/>
       <c r="S47" s="21"/>
@@ -7890,7 +7899,7 @@
         <v>30</v>
       </c>
       <c r="AB47" s="200" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="AC47" s="126" t="s">
         <v>30</v>
@@ -7898,7 +7907,7 @@
       <c r="AD47" s="21"/>
       <c r="AE47" s="21"/>
       <c r="AF47" s="98" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="AG47" s="103" t="s">
         <v>30</v>
@@ -7946,7 +7955,7 @@
       <c r="G48" s="21"/>
       <c r="H48" s="21"/>
       <c r="I48" s="98" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="J48" s="103"/>
       <c r="K48" s="21"/>
@@ -8034,7 +8043,7 @@
       <c r="H49" s="103"/>
       <c r="I49" s="21"/>
       <c r="J49" s="21" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="K49" s="21"/>
       <c r="L49" s="21"/>
@@ -8383,7 +8392,7 @@
       </c>
       <c r="P53" s="21"/>
       <c r="Q53" s="126" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="R53" s="22" t="s">
         <v>30</v>
@@ -8486,7 +8495,7 @@
       <c r="Y54" s="103"/>
       <c r="Z54" s="21"/>
       <c r="AA54" s="98" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="AB54" s="21"/>
       <c r="AC54" s="126" t="s">
@@ -8691,12 +8700,14 @@
         <v>159</v>
       </c>
       <c r="B57" s="208" t="s">
+        <v>518</v>
+      </c>
+      <c r="C57" s="76" t="s">
         <v>519</v>
       </c>
-      <c r="C57" s="76" t="s">
-        <v>520</v>
-      </c>
-      <c r="D57" s="76"/>
+      <c r="D57" s="76" t="s">
+        <v>529</v>
+      </c>
       <c r="E57" s="43">
         <f t="shared" si="4"/>
         <v>4</v>
@@ -8756,12 +8767,14 @@
         <v>160</v>
       </c>
       <c r="B58" s="209" t="s">
-        <v>521</v>
+        <v>354</v>
       </c>
       <c r="C58" s="72" t="s">
-        <v>522</v>
-      </c>
-      <c r="D58" s="72"/>
+        <v>116</v>
+      </c>
+      <c r="D58" s="72" t="s">
+        <v>98</v>
+      </c>
       <c r="E58" s="73">
         <f t="shared" si="4"/>
         <v>6</v>
@@ -8817,7 +8830,7 @@
       </c>
       <c r="AN58" s="12" t="str">
         <f t="shared" si="6"/>
-        <v>David  Conway-Holland</v>
+        <v>Thomas Jeremy Ward</v>
       </c>
     </row>
     <row r="59" spans="1:51" ht="15" customHeight="1" x14ac:dyDescent="0.15">
@@ -8825,12 +8838,14 @@
         <v>161</v>
       </c>
       <c r="B59" s="26" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
       <c r="C59" s="26" t="s">
-        <v>524</v>
-      </c>
-      <c r="D59" s="26"/>
+        <v>521</v>
+      </c>
+      <c r="D59" s="26" t="s">
+        <v>528</v>
+      </c>
       <c r="E59" s="43">
         <f t="shared" si="4"/>
         <v>7</v>
@@ -8895,9 +8910,15 @@
       <c r="A60" s="59" t="s">
         <v>162</v>
       </c>
-      <c r="B60" s="26"/>
-      <c r="C60" s="26"/>
-      <c r="D60" s="26"/>
+      <c r="B60" s="12" t="s">
+        <v>525</v>
+      </c>
+      <c r="C60" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="D60" s="26" t="s">
+        <v>526</v>
+      </c>
       <c r="E60" s="43">
         <f t="shared" si="4"/>
         <v>8</v>
@@ -8956,8 +8977,8 @@
         <v>8</v>
       </c>
       <c r="AN60" s="12" t="str">
-        <f t="shared" ref="AN60:AN62" si="7">B60&amp;" "&amp;C60</f>
-        <v xml:space="preserve"> </v>
+        <f>B61&amp;" "&amp;C61</f>
+        <v>Nasser Sharifi</v>
       </c>
     </row>
     <row r="61" spans="1:51" s="28" customFormat="1" ht="14" x14ac:dyDescent="0.15">
@@ -8965,12 +8986,14 @@
         <v>163</v>
       </c>
       <c r="B61" s="26" t="s">
-        <v>43</v>
-      </c>
-      <c r="C61" s="27" t="s">
-        <v>518</v>
-      </c>
-      <c r="D61" s="26"/>
+        <v>523</v>
+      </c>
+      <c r="C61" s="26" t="s">
+        <v>524</v>
+      </c>
+      <c r="D61" s="28" t="s">
+        <v>527</v>
+      </c>
       <c r="E61" s="43">
         <f t="shared" si="4"/>
         <v>5</v>
@@ -9023,7 +9046,7 @@
         <v>5</v>
       </c>
       <c r="AN61" s="12" t="str">
-        <f t="shared" si="7"/>
+        <f>B62&amp;" "&amp;C62</f>
         <v>David Hilton MBE, RN</v>
       </c>
       <c r="AY61" s="12"/>
@@ -9033,12 +9056,14 @@
         <v>111</v>
       </c>
       <c r="B62" s="26" t="s">
-        <v>525</v>
-      </c>
-      <c r="C62" s="26" t="s">
-        <v>526</v>
-      </c>
-      <c r="D62" s="26"/>
+        <v>43</v>
+      </c>
+      <c r="C62" s="27" t="s">
+        <v>517</v>
+      </c>
+      <c r="D62" s="26" t="s">
+        <v>59</v>
+      </c>
       <c r="E62" s="43">
         <f t="shared" si="4"/>
         <v>7</v>
@@ -9094,9 +9119,9 @@
         <f t="shared" si="5"/>
         <v>7</v>
       </c>
-      <c r="AN62" s="12" t="str">
-        <f t="shared" si="7"/>
-        <v>Brett Clark</v>
+      <c r="AN62" s="12" t="e">
+        <f>#REF!&amp;" "&amp;#REF!</f>
+        <v>#REF!</v>
       </c>
     </row>
   </sheetData>
@@ -9128,13 +9153,13 @@
   <sheetData>
     <row r="3" spans="4:19" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D3" s="124" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="E3" s="116" t="s">
         <v>221</v>
       </c>
       <c r="F3" s="116" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="G3" s="116" t="s">
         <v>222</v>
@@ -9223,13 +9248,13 @@
         <v>240</v>
       </c>
       <c r="P5" s="196" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="R5" s="166" t="s">
         <v>14</v>
       </c>
       <c r="S5" s="181" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
     </row>
     <row r="6" spans="4:19" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -9265,10 +9290,10 @@
         <v>247</v>
       </c>
       <c r="R6" s="166" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="S6" s="178" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="7" spans="4:19" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -9302,10 +9327,10 @@
         <v>254</v>
       </c>
       <c r="R7" s="168" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="S7" s="179" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
     </row>
     <row r="8" spans="4:19" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -9341,10 +9366,10 @@
         <v>262</v>
       </c>
       <c r="R8" s="167" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="S8" s="180" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
     </row>
     <row r="9" spans="4:19" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -9382,7 +9407,7 @@
         <v>269</v>
       </c>
       <c r="R9" s="168" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="S9" s="179" t="s">
         <v>240</v>
@@ -9648,7 +9673,7 @@
         <v>321</v>
       </c>
       <c r="P17" s="195" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
     </row>
     <row r="18" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -9697,20 +9722,20 @@
         <v>250</v>
       </c>
       <c r="I19" s="117" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="J19" s="117" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="K19" s="118"/>
       <c r="L19" s="117" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="M19" s="121" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="N19" s="117" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
     </row>
     <row r="20" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -9746,7 +9771,7 @@
         <v>334</v>
       </c>
       <c r="P20" s="195" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
     </row>
     <row r="21" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -9764,7 +9789,7 @@
         <v>336</v>
       </c>
       <c r="I21" s="118" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="J21" s="117" t="s">
         <v>232</v>
@@ -9861,22 +9886,22 @@
         <v>356</v>
       </c>
       <c r="I24" s="160" t="s">
-        <v>357</v>
+        <v>522</v>
       </c>
       <c r="J24" s="160" t="s">
         <v>232</v>
       </c>
       <c r="K24" s="160" t="s">
+        <v>357</v>
+      </c>
+      <c r="L24" s="160" t="s">
         <v>358</v>
       </c>
-      <c r="L24" s="160" t="s">
+      <c r="M24" s="160" t="s">
         <v>359</v>
       </c>
-      <c r="M24" s="160" t="s">
+      <c r="N24" s="160" t="s">
         <v>360</v>
-      </c>
-      <c r="N24" s="160" t="s">
-        <v>361</v>
       </c>
     </row>
     <row r="25" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -9887,27 +9912,27 @@
         <v>200</v>
       </c>
       <c r="F25" s="117" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="G25" s="118"/>
       <c r="H25" s="117" t="s">
+        <v>362</v>
+      </c>
+      <c r="I25" s="117" t="s">
         <v>363</v>
-      </c>
-      <c r="I25" s="117" t="s">
-        <v>364</v>
       </c>
       <c r="J25" s="117" t="s">
         <v>232</v>
       </c>
       <c r="K25" s="118"/>
       <c r="L25" s="117" t="s">
+        <v>364</v>
+      </c>
+      <c r="M25" s="117" t="s">
         <v>365</v>
       </c>
-      <c r="M25" s="117" t="s">
+      <c r="N25" s="117" t="s">
         <v>366</v>
-      </c>
-      <c r="N25" s="117" t="s">
-        <v>367</v>
       </c>
     </row>
     <row r="26" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -9918,27 +9943,27 @@
         <v>201</v>
       </c>
       <c r="F26" s="157" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="G26" s="158"/>
       <c r="H26" s="157" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="I26" s="157" t="s">
         <v>324</v>
       </c>
       <c r="J26" s="157" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="K26" s="158"/>
       <c r="L26" s="157" t="s">
+        <v>370</v>
+      </c>
+      <c r="M26" s="157" t="s">
         <v>371</v>
       </c>
-      <c r="M26" s="157" t="s">
+      <c r="N26" s="157" t="s">
         <v>372</v>
-      </c>
-      <c r="N26" s="157" t="s">
-        <v>373</v>
       </c>
     </row>
     <row r="27" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -9949,29 +9974,29 @@
         <v>202</v>
       </c>
       <c r="F27" s="150" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="G27" s="151"/>
       <c r="H27" s="150" t="s">
+        <v>374</v>
+      </c>
+      <c r="I27" s="150" t="s">
         <v>375</v>
-      </c>
-      <c r="I27" s="150" t="s">
-        <v>376</v>
       </c>
       <c r="J27" s="150" t="s">
         <v>232</v>
       </c>
       <c r="K27" s="150" t="s">
+        <v>376</v>
+      </c>
+      <c r="L27" s="150" t="s">
         <v>377</v>
       </c>
-      <c r="L27" s="150" t="s">
+      <c r="M27" s="150" t="s">
         <v>378</v>
       </c>
-      <c r="M27" s="150" t="s">
+      <c r="N27" s="150" t="s">
         <v>379</v>
-      </c>
-      <c r="N27" s="150" t="s">
-        <v>380</v>
       </c>
     </row>
     <row r="28" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -9982,7 +10007,7 @@
         <v>61</v>
       </c>
       <c r="F28" s="117" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="G28" s="118"/>
       <c r="H28" s="117" t="s">
@@ -9995,16 +10020,16 @@
         <v>232</v>
       </c>
       <c r="K28" s="117" t="s">
+        <v>381</v>
+      </c>
+      <c r="L28" s="117" t="s">
         <v>382</v>
       </c>
-      <c r="L28" s="117" t="s">
+      <c r="M28" s="117" t="s">
         <v>383</v>
       </c>
-      <c r="M28" s="117" t="s">
+      <c r="N28" s="117" t="s">
         <v>384</v>
-      </c>
-      <c r="N28" s="117" t="s">
-        <v>385</v>
       </c>
     </row>
     <row r="29" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -10012,14 +10037,14 @@
         <v>100</v>
       </c>
       <c r="E29" s="117" t="s">
+        <v>385</v>
+      </c>
+      <c r="F29" s="117" t="s">
         <v>386</v>
-      </c>
-      <c r="F29" s="117" t="s">
-        <v>387</v>
       </c>
       <c r="G29" s="118"/>
       <c r="H29" s="117" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="I29" s="117" t="s">
         <v>81</v>
@@ -10028,16 +10053,16 @@
         <v>232</v>
       </c>
       <c r="K29" s="117" t="s">
+        <v>388</v>
+      </c>
+      <c r="L29" s="117" t="s">
+        <v>388</v>
+      </c>
+      <c r="M29" s="117" t="s">
         <v>389</v>
       </c>
-      <c r="L29" s="117" t="s">
-        <v>389</v>
-      </c>
-      <c r="M29" s="117" t="s">
+      <c r="N29" s="117" t="s">
         <v>390</v>
-      </c>
-      <c r="N29" s="117" t="s">
-        <v>391</v>
       </c>
     </row>
     <row r="30" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -10048,11 +10073,11 @@
         <v>97</v>
       </c>
       <c r="F30" s="157" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="G30" s="158"/>
       <c r="H30" s="157" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="I30" s="157" t="s">
         <v>97</v>
@@ -10061,16 +10086,16 @@
         <v>232</v>
       </c>
       <c r="K30" s="157" t="s">
+        <v>393</v>
+      </c>
+      <c r="L30" s="157" t="s">
         <v>394</v>
       </c>
-      <c r="L30" s="157" t="s">
+      <c r="M30" s="157" t="s">
         <v>395</v>
       </c>
-      <c r="M30" s="157" t="s">
+      <c r="N30" s="157" t="s">
         <v>396</v>
-      </c>
-      <c r="N30" s="157" t="s">
-        <v>397</v>
       </c>
     </row>
     <row r="31" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -10081,29 +10106,29 @@
         <v>203</v>
       </c>
       <c r="F31" s="117" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="G31" s="118"/>
       <c r="H31" s="117" t="s">
+        <v>398</v>
+      </c>
+      <c r="I31" s="117" t="s">
         <v>399</v>
-      </c>
-      <c r="I31" s="117" t="s">
-        <v>400</v>
       </c>
       <c r="J31" s="117" t="s">
         <v>232</v>
       </c>
       <c r="K31" s="117" t="s">
+        <v>400</v>
+      </c>
+      <c r="L31" s="117" t="s">
         <v>401</v>
       </c>
-      <c r="L31" s="117" t="s">
+      <c r="M31" s="117" t="s">
         <v>402</v>
       </c>
-      <c r="M31" s="117" t="s">
+      <c r="N31" s="117" t="s">
         <v>403</v>
-      </c>
-      <c r="N31" s="117" t="s">
-        <v>404</v>
       </c>
     </row>
     <row r="32" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -10114,29 +10139,29 @@
         <v>204</v>
       </c>
       <c r="F32" s="160" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="G32" s="161"/>
       <c r="H32" s="160" t="s">
+        <v>405</v>
+      </c>
+      <c r="I32" s="160" t="s">
         <v>406</v>
-      </c>
-      <c r="I32" s="160" t="s">
-        <v>407</v>
       </c>
       <c r="J32" s="160" t="s">
         <v>232</v>
       </c>
       <c r="K32" s="160" t="s">
+        <v>407</v>
+      </c>
+      <c r="L32" s="160" t="s">
         <v>408</v>
       </c>
-      <c r="L32" s="160" t="s">
+      <c r="M32" s="160" t="s">
         <v>409</v>
       </c>
-      <c r="M32" s="160" t="s">
+      <c r="N32" s="160" t="s">
         <v>410</v>
-      </c>
-      <c r="N32" s="160" t="s">
-        <v>411</v>
       </c>
     </row>
     <row r="33" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -10144,14 +10169,14 @@
         <v>105</v>
       </c>
       <c r="E33" s="117" t="s">
+        <v>485</v>
+      </c>
+      <c r="F33" s="117" t="s">
         <v>486</v>
-      </c>
-      <c r="F33" s="117" t="s">
-        <v>487</v>
       </c>
       <c r="G33" s="118"/>
       <c r="H33" s="117" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="I33" s="117" t="s">
         <v>99</v>
@@ -10160,16 +10185,16 @@
         <v>232</v>
       </c>
       <c r="K33" s="117" t="s">
+        <v>488</v>
+      </c>
+      <c r="L33" s="117" t="s">
         <v>489</v>
       </c>
-      <c r="L33" s="117" t="s">
+      <c r="M33" s="117" t="s">
         <v>490</v>
       </c>
-      <c r="M33" s="117" t="s">
+      <c r="N33" s="117" t="s">
         <v>491</v>
-      </c>
-      <c r="N33" s="117" t="s">
-        <v>492</v>
       </c>
     </row>
     <row r="34" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -10180,29 +10205,29 @@
         <v>205</v>
       </c>
       <c r="F34" s="153" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="G34" s="154"/>
       <c r="H34" s="153" t="s">
+        <v>412</v>
+      </c>
+      <c r="I34" s="153" t="s">
         <v>413</v>
-      </c>
-      <c r="I34" s="153" t="s">
-        <v>414</v>
       </c>
       <c r="J34" s="153" t="s">
         <v>232</v>
       </c>
       <c r="K34" s="153" t="s">
+        <v>414</v>
+      </c>
+      <c r="L34" s="153" t="s">
         <v>415</v>
       </c>
-      <c r="L34" s="153" t="s">
+      <c r="M34" s="153" t="s">
         <v>416</v>
       </c>
-      <c r="M34" s="153" t="s">
+      <c r="N34" s="153" t="s">
         <v>417</v>
-      </c>
-      <c r="N34" s="153" t="s">
-        <v>418</v>
       </c>
     </row>
     <row r="35" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -10213,29 +10238,29 @@
         <v>206</v>
       </c>
       <c r="F35" s="150" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="G35" s="151"/>
       <c r="H35" s="150" t="s">
+        <v>419</v>
+      </c>
+      <c r="I35" s="150" t="s">
         <v>420</v>
-      </c>
-      <c r="I35" s="150" t="s">
-        <v>421</v>
       </c>
       <c r="J35" s="150" t="s">
         <v>232</v>
       </c>
       <c r="K35" s="150" t="s">
+        <v>421</v>
+      </c>
+      <c r="L35" s="150" t="s">
         <v>422</v>
       </c>
-      <c r="L35" s="150" t="s">
+      <c r="M35" s="150" t="s">
         <v>423</v>
       </c>
-      <c r="M35" s="150" t="s">
+      <c r="N35" s="150" t="s">
         <v>424</v>
-      </c>
-      <c r="N35" s="150" t="s">
-        <v>425</v>
       </c>
     </row>
     <row r="36" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -10246,30 +10271,30 @@
         <v>207</v>
       </c>
       <c r="F36" s="157" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="G36" s="158"/>
       <c r="H36" s="157" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="I36" s="157" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="J36" s="157" t="s">
         <v>232</v>
       </c>
       <c r="K36" s="158"/>
       <c r="L36" s="157" t="s">
+        <v>427</v>
+      </c>
+      <c r="M36" s="157" t="s">
         <v>428</v>
       </c>
-      <c r="M36" s="157" t="s">
+      <c r="N36" s="157" t="s">
         <v>429</v>
       </c>
-      <c r="N36" s="157" t="s">
-        <v>430</v>
-      </c>
       <c r="P36" s="196" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="37" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -10280,29 +10305,29 @@
         <v>208</v>
       </c>
       <c r="F37" s="157" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="G37" s="158"/>
       <c r="H37" s="157" t="s">
+        <v>431</v>
+      </c>
+      <c r="I37" s="157" t="s">
         <v>432</v>
-      </c>
-      <c r="I37" s="157" t="s">
-        <v>433</v>
       </c>
       <c r="J37" s="157" t="s">
         <v>232</v>
       </c>
       <c r="K37" s="157" t="s">
+        <v>433</v>
+      </c>
+      <c r="L37" s="157" t="s">
         <v>434</v>
       </c>
-      <c r="L37" s="157" t="s">
+      <c r="M37" s="157" t="s">
         <v>435</v>
       </c>
-      <c r="M37" s="157" t="s">
+      <c r="N37" s="157" t="s">
         <v>436</v>
-      </c>
-      <c r="N37" s="157" t="s">
-        <v>437</v>
       </c>
     </row>
     <row r="38" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -10313,29 +10338,29 @@
         <v>209</v>
       </c>
       <c r="F38" s="170" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="G38" s="171"/>
       <c r="H38" s="170" t="s">
+        <v>438</v>
+      </c>
+      <c r="I38" s="170" t="s">
         <v>439</v>
-      </c>
-      <c r="I38" s="170" t="s">
-        <v>440</v>
       </c>
       <c r="J38" s="170" t="s">
         <v>232</v>
       </c>
       <c r="K38" s="170" t="s">
+        <v>440</v>
+      </c>
+      <c r="L38" s="170" t="s">
         <v>441</v>
       </c>
-      <c r="L38" s="170" t="s">
+      <c r="M38" s="170" t="s">
         <v>442</v>
       </c>
-      <c r="M38" s="170" t="s">
+      <c r="N38" s="170" t="s">
         <v>443</v>
-      </c>
-      <c r="N38" s="170" t="s">
-        <v>444</v>
       </c>
     </row>
     <row r="39" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -10346,32 +10371,32 @@
         <v>210</v>
       </c>
       <c r="F39" s="157" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="G39" s="158"/>
       <c r="H39" s="157" t="s">
         <v>330</v>
       </c>
       <c r="I39" s="157" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="J39" s="157" t="s">
         <v>232</v>
       </c>
       <c r="K39" s="157" t="s">
+        <v>446</v>
+      </c>
+      <c r="L39" s="157" t="s">
         <v>447</v>
       </c>
-      <c r="L39" s="157" t="s">
+      <c r="M39" s="157" t="s">
         <v>448</v>
       </c>
-      <c r="M39" s="157" t="s">
+      <c r="N39" s="157" t="s">
         <v>449</v>
       </c>
-      <c r="N39" s="157" t="s">
-        <v>450</v>
-      </c>
       <c r="P39" s="196" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
     </row>
     <row r="40" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -10382,27 +10407,27 @@
         <v>211</v>
       </c>
       <c r="F40" s="150" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="G40" s="151"/>
       <c r="H40" s="150" t="s">
+        <v>451</v>
+      </c>
+      <c r="I40" s="150" t="s">
         <v>452</v>
-      </c>
-      <c r="I40" s="150" t="s">
-        <v>453</v>
       </c>
       <c r="J40" s="150" t="s">
         <v>232</v>
       </c>
       <c r="K40" s="151"/>
       <c r="L40" s="150" t="s">
+        <v>453</v>
+      </c>
+      <c r="M40" s="150" t="s">
         <v>454</v>
       </c>
-      <c r="M40" s="150" t="s">
+      <c r="N40" s="150" t="s">
         <v>455</v>
-      </c>
-      <c r="N40" s="150" t="s">
-        <v>456</v>
       </c>
     </row>
     <row r="41" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -10413,32 +10438,32 @@
         <v>212</v>
       </c>
       <c r="F41" s="150" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="G41" s="151"/>
       <c r="H41" s="150" t="s">
+        <v>457</v>
+      </c>
+      <c r="I41" s="150" t="s">
         <v>458</v>
-      </c>
-      <c r="I41" s="150" t="s">
-        <v>459</v>
       </c>
       <c r="J41" s="150" t="s">
         <v>232</v>
       </c>
       <c r="K41" s="150" t="s">
+        <v>459</v>
+      </c>
+      <c r="L41" s="150" t="s">
         <v>460</v>
       </c>
-      <c r="L41" s="150" t="s">
+      <c r="M41" s="150" t="s">
         <v>461</v>
       </c>
-      <c r="M41" s="150" t="s">
+      <c r="N41" s="150" t="s">
         <v>462</v>
       </c>
-      <c r="N41" s="150" t="s">
-        <v>463</v>
-      </c>
       <c r="P41" s="201" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
     </row>
     <row r="42" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -10449,7 +10474,7 @@
         <v>213</v>
       </c>
       <c r="F42" s="117" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="G42" s="118"/>
       <c r="H42" s="117" t="s">
@@ -10462,16 +10487,16 @@
         <v>232</v>
       </c>
       <c r="K42" s="117" t="s">
+        <v>464</v>
+      </c>
+      <c r="L42" s="117" t="s">
         <v>465</v>
       </c>
-      <c r="L42" s="117" t="s">
+      <c r="M42" s="117" t="s">
         <v>466</v>
       </c>
-      <c r="M42" s="117" t="s">
+      <c r="N42" s="117" t="s">
         <v>467</v>
-      </c>
-      <c r="N42" s="117" t="s">
-        <v>468</v>
       </c>
     </row>
     <row r="43" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -10482,29 +10507,29 @@
         <v>214</v>
       </c>
       <c r="F43" s="117" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="G43" s="118"/>
       <c r="H43" s="117" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="I43" s="117" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="J43" s="117" t="s">
         <v>232</v>
       </c>
       <c r="K43" s="117" t="s">
+        <v>470</v>
+      </c>
+      <c r="L43" s="117" t="s">
         <v>471</v>
       </c>
-      <c r="L43" s="117" t="s">
+      <c r="M43" s="117" t="s">
         <v>472</v>
       </c>
-      <c r="M43" s="117" t="s">
+      <c r="N43" s="117" t="s">
         <v>473</v>
-      </c>
-      <c r="N43" s="117" t="s">
-        <v>474</v>
       </c>
     </row>
     <row r="44" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -10515,11 +10540,11 @@
         <v>215</v>
       </c>
       <c r="F44" s="117" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="G44" s="118"/>
       <c r="H44" s="117" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="I44" s="118"/>
       <c r="J44" s="117" t="s">
@@ -10527,13 +10552,13 @@
       </c>
       <c r="K44" s="118"/>
       <c r="L44" s="117" t="s">
+        <v>476</v>
+      </c>
+      <c r="M44" s="117" t="s">
         <v>477</v>
       </c>
-      <c r="M44" s="117" t="s">
+      <c r="N44" s="117" t="s">
         <v>478</v>
-      </c>
-      <c r="N44" s="117" t="s">
-        <v>479</v>
       </c>
     </row>
     <row r="45" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -10544,11 +10569,11 @@
         <v>216</v>
       </c>
       <c r="F45" s="191" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="G45" s="192"/>
       <c r="H45" s="191" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="I45" s="191" t="s">
         <v>324</v>
@@ -10557,16 +10582,16 @@
         <v>232</v>
       </c>
       <c r="K45" s="191" t="s">
+        <v>481</v>
+      </c>
+      <c r="L45" s="191" t="s">
         <v>482</v>
       </c>
-      <c r="L45" s="191" t="s">
+      <c r="M45" s="191" t="s">
         <v>483</v>
       </c>
-      <c r="M45" s="191" t="s">
+      <c r="N45" s="191" t="s">
         <v>484</v>
-      </c>
-      <c r="N45" s="191" t="s">
-        <v>485</v>
       </c>
     </row>
     <row r="46" spans="4:16" x14ac:dyDescent="0.15">

</xml_diff>

<commit_message>
feat: allow for inactive officers in the list
</commit_message>
<xml_diff>
--- a/samples/ra/26-27/Royal Arch Official Visit Matrix 2026 - 2027 MF V5 04082026.xlsx
+++ b/samples/ra/26-27/Royal Arch Official Visit Matrix 2026 - 2027 MF V5 04082026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kpturner/github/square_ov/samples/ra/26-27/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC4A4D1B-9B8E-9349-BF8C-1D3E8D833FA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9A5D73C-D7A7-924F-A1CB-62DDF1895B1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30520" yWindow="29360" windowWidth="34360" windowHeight="19800" tabRatio="500" activeTab="1" xr2:uid="{FA0C5B21-D744-41D8-A854-64181BC35FE8}"/>
+    <workbookView xWindow="30520" yWindow="29360" windowWidth="34360" windowHeight="19800" tabRatio="500" xr2:uid="{FA0C5B21-D744-41D8-A854-64181BC35FE8}"/>
   </bookViews>
   <sheets>
     <sheet name="2026-2027 Official Visits" sheetId="1" r:id="rId1"/>
@@ -2484,7 +2484,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="26">
+  <borders count="27">
     <border>
       <left/>
       <right/>
@@ -2801,6 +2801,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="8"/>
+      </right>
+      <top style="thin">
+        <color indexed="8"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="8"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -2848,7 +2863,7 @@
     <xf numFmtId="0" fontId="1" fillId="36" borderId="20" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="41" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="210">
+  <cellXfs count="211">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
@@ -3421,6 +3436,7 @@
     <xf numFmtId="0" fontId="49" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="44">
     <cellStyle name="20% - Accent1" xfId="18" builtinId="30" customBuiltin="1"/>
@@ -8913,7 +8929,7 @@
       <c r="B60" s="12" t="s">
         <v>525</v>
       </c>
-      <c r="C60" s="12" t="s">
+      <c r="C60" s="210" t="s">
         <v>40</v>
       </c>
       <c r="D60" s="26" t="s">

</xml_diff>